<commit_message>
feat: 39 named ranges colonnes + check_marks via ref_range (élimination START/END)
</commit_message>
<xml_diff>
--- a/comptes_exemple.xlsx
+++ b/comptes_exemple.xlsx
@@ -17,15 +17,30 @@
   </sheets>
   <definedNames>
     <definedName name="année_courante" hidden="0" function="0" vbProcedure="0">Avoirs!$A$1</definedName>
+    <definedName name="AVRdate_anter" hidden="0" function="0" vbProcedure="0">Avoirs!$H$4:$H$31</definedName>
     <definedName name="AVRdate_solde" hidden="0" function="0" vbProcedure="0">Avoirs!$J$4:$J$31</definedName>
+    <definedName name="AVRdevise" hidden="0" function="0" vbProcedure="0">Avoirs!$E$4:$E$31</definedName>
     <definedName name="AVRdomiciliation" hidden="0" function="0" vbProcedure="0">Avoirs!$C$4:$C$31</definedName>
     <definedName name="AVRintitulé" hidden="0" function="0" vbProcedure="0">Avoirs!$A$4:$A$31</definedName>
+    <definedName name="AVRmontant_anter" hidden="0" function="0" vbProcedure="0">Avoirs!$I$4:$I$31</definedName>
     <definedName name="AVRmontant_solde" hidden="0" function="0" vbProcedure="0">Avoirs!$K$4:$K$31</definedName>
     <definedName name="AVRmontant_solde_euro" hidden="0" function="0" vbProcedure="0">Avoirs!$L$4:$L$31</definedName>
     <definedName name="AVRpropriete" hidden="0" function="0" vbProcedure="0">Avoirs!$G$4:$G$31</definedName>
     <definedName name="AVRsous_type" hidden="0" function="0" vbProcedure="0">Avoirs!$D$4:$D$31</definedName>
     <definedName name="AVRtitulaire" hidden="0" function="0" vbProcedure="0">Avoirs!$F$4:$F$31</definedName>
     <definedName name="AVRtype" hidden="0" function="0" vbProcedure="0">Avoirs!$B$4:$B$31</definedName>
+    <definedName name="CATaffectation" hidden="0" function="0" vbProcedure="0">Budget!$P$19:$P$35</definedName>
+    <definedName name="CATaffectation_pct" hidden="0" function="0" vbProcedure="0">Budget!$O$19:$O$35</definedName>
+    <definedName name="CATnom" hidden="0" function="0" vbProcedure="0">Budget!$E$19:$E$35</definedName>
+    <definedName name="CATposte" hidden="0" function="0" vbProcedure="0">Budget!$Q$19:$Q$35</definedName>
+    <definedName name="CATtotal_euro" hidden="0" function="0" vbProcedure="0">Budget!$N$19:$N$35</definedName>
+    <definedName name="COTcode" hidden="0" function="0" vbProcedure="0">Cotations!$E$3:$E$12</definedName>
+    <definedName name="COTcours" hidden="0" function="0" vbProcedure="0">Cotations!$F$3:$F$12</definedName>
+    <definedName name="COTdate" hidden="0" function="0" vbProcedure="0">Cotations!$G$3:$G$12</definedName>
+    <definedName name="COTdecimales" hidden="0" function="0" vbProcedure="0">Cotations!$D$3:$D$12</definedName>
+    <definedName name="COTfamille" hidden="0" function="0" vbProcedure="0">Cotations!$C$3:$C$12</definedName>
+    <definedName name="COTlabel" hidden="0" function="0" vbProcedure="0">Cotations!$A$3:$A$12</definedName>
+    <definedName name="COTnature" hidden="0" function="0" vbProcedure="0">Cotations!$B$3:$B$12</definedName>
     <definedName name="Cours_AgPr" hidden="0" function="0" vbProcedure="0">#REF!</definedName>
     <definedName name="cours_BTC" hidden="0" function="0" vbProcedure="0">Cotations!$F$7</definedName>
     <definedName name="cours_OrPr" hidden="0" function="0" vbProcedure="0">Cotations!$F$6</definedName>
@@ -34,6 +49,18 @@
     <definedName name="cours_USD" hidden="0" function="0" vbProcedure="0">Cotations!$F$10</definedName>
     <definedName name="cours_XAU" hidden="0" function="0" vbProcedure="0">Cotations!$F$5</definedName>
     <definedName name="cours_XMR" hidden="0" function="0" vbProcedure="0">Cotations!$F$9</definedName>
+    <definedName name="CTRL1compte" hidden="0" function="0" vbProcedure="0">Contrôles!$A$3:$A$26</definedName>
+    <definedName name="CTRL1controle" hidden="0" function="0" vbProcedure="0">Contrôles!$I$3:$I$26</definedName>
+    <definedName name="CTRL1date_ancrage" hidden="0" function="0" vbProcedure="0">Contrôles!$C$3:$C$26</definedName>
+    <definedName name="CTRL1date_releve" hidden="0" function="0" vbProcedure="0">Contrôles!$D$3:$D$26</definedName>
+    <definedName name="CTRL1devise" hidden="0" function="0" vbProcedure="0">Contrôles!$B$3:$B$26</definedName>
+    <definedName name="CTRL1ecart" hidden="0" function="0" vbProcedure="0">Contrôles!$H$3:$H$26</definedName>
+    <definedName name="CTRL1montant_ancrage" hidden="0" function="0" vbProcedure="0">Contrôles!$E$3:$E$26</definedName>
+    <definedName name="CTRL1montant_releve" hidden="0" function="0" vbProcedure="0">Contrôles!$G$3:$G$26</definedName>
+    <definedName name="CTRL1solde_calc" hidden="0" function="0" vbProcedure="0">Contrôles!$F$3:$F$26</definedName>
+    <definedName name="CTRL2affichage" hidden="0" function="0" vbProcedure="0">Contrôles!$K$32:$K$44</definedName>
+    <definedName name="CTRL2general" hidden="0" function="0" vbProcedure="0">Contrôles!$L$32:$L$44</definedName>
+    <definedName name="CTRL2type" hidden="0" function="0" vbProcedure="0">Contrôles!$J$32:$J$44</definedName>
     <definedName name="END_AVR" hidden="0" function="0" vbProcedure="0">Avoirs!$A$31</definedName>
     <definedName name="END_CAT" hidden="0" function="0" vbProcedure="0">Budget!$E$35</definedName>
     <definedName name="END_COT" hidden="0" function="0" vbProcedure="0">Cotations!$A$12</definedName>
@@ -43,6 +70,7 @@
     <definedName name="END_POSTES" hidden="0" function="0" vbProcedure="0">Budget!$A$10</definedName>
     <definedName name="END_PVL" hidden="0" function="0" vbProcedure="0">Plus_value!$B$52</definedName>
     <definedName name="OPcatégorie" hidden="0" function="0" vbProcedure="0">Opérations!$G$4:$G$10000</definedName>
+    <definedName name="OPcommentaire" hidden="0" function="0" vbProcedure="0">Opérations!$I$4:$I$7193</definedName>
     <definedName name="OPcompte" hidden="0" function="0" vbProcedure="0">Opérations!$H$4:$H$10000</definedName>
     <definedName name="OPdate" hidden="0" function="0" vbProcedure="0">Opérations!$A$4:$A$10000</definedName>
     <definedName name="OPdevise" hidden="0" function="0" vbProcedure="0">Opérations!$D$4:$D$10000</definedName>
@@ -50,9 +78,21 @@
     <definedName name="OPlibellé" hidden="0" function="0" vbProcedure="0">Opérations!$B$4:$B$10000</definedName>
     <definedName name="OPmontant" hidden="0" function="0" vbProcedure="0">Opérations!$C$4:$C$10000</definedName>
     <definedName name="OPréf" hidden="0" function="0" vbProcedure="0">Opérations!$F$4:$F$10000</definedName>
+    <definedName name="PATlabel" hidden="0" function="0" vbProcedure="0">Patrimoine!$B$5:$B$51</definedName>
+    <definedName name="PATnombre" hidden="0" function="0" vbProcedure="0">Patrimoine!$C$5:$C$51</definedName>
+    <definedName name="PATpoids" hidden="0" function="0" vbProcedure="0">Patrimoine!$E$5:$E$51</definedName>
+    <definedName name="PATvaleur" hidden="0" function="0" vbProcedure="0">Patrimoine!$D$5:$D$51</definedName>
+    <definedName name="POSTESnom" hidden="0" function="0" vbProcedure="0">Budget!$A$4:$A$10</definedName>
     <definedName name="PVLcompte" hidden="0" function="0" vbProcedure="0">Plus_value!$B$5:$B$52</definedName>
     <definedName name="PVLdate" hidden="0" function="0" vbProcedure="0">Plus_value!$J$5:$J$52</definedName>
+    <definedName name="PVLdate_init" hidden="0" function="0" vbProcedure="0">Plus_value!$G$5:$G$52</definedName>
+    <definedName name="PVLdevise" hidden="0" function="0" vbProcedure="0">Plus_value!$D$5:$D$52</definedName>
     <definedName name="PVLmontant" hidden="0" function="0" vbProcedure="0">Plus_value!$K$5:$K$52</definedName>
+    <definedName name="PVLmontant_init" hidden="0" function="0" vbProcedure="0">Plus_value!$H$5:$H$52</definedName>
+    <definedName name="PVLpct" hidden="0" function="0" vbProcedure="0">Plus_value!$F$5:$F$52</definedName>
+    <definedName name="PVLpvl" hidden="0" function="0" vbProcedure="0">Plus_value!$E$5:$E$52</definedName>
+    <definedName name="PVLsection" hidden="0" function="0" vbProcedure="0">Plus_value!$A$5:$A$52</definedName>
+    <definedName name="PVLsigma" hidden="0" function="0" vbProcedure="0">Plus_value!$I$5:$I$52</definedName>
     <definedName name="PVLtitre" hidden="0" function="0" vbProcedure="0">Plus_value!$C$5:$C$52</definedName>
     <definedName name="Retenu" hidden="0" function="0" vbProcedure="0">"Retenu"</definedName>
     <definedName name="Solde" hidden="0" function="0" vbProcedure="0">"#Solde"</definedName>

</xml_diff>

<commit_message>
feat: CTRL2eur named range + suppression offsets +3 dans gui_devises/tool_template
</commit_message>
<xml_diff>
--- a/comptes_exemple.xlsx
+++ b/comptes_exemple.xlsx
@@ -59,6 +59,7 @@
     <definedName name="CTRL1montant_releve" hidden="0" function="0" vbProcedure="0">Contrôles!$G$3:$G$26</definedName>
     <definedName name="CTRL1solde_calc" hidden="0" function="0" vbProcedure="0">Contrôles!$F$3:$F$26</definedName>
     <definedName name="CTRL2affichage" hidden="0" function="0" vbProcedure="0">Contrôles!$K$32:$K$44</definedName>
+    <definedName name="CTRL2eur" hidden="0" function="0" vbProcedure="0">Contrôles!$M$32:$M$44</definedName>
     <definedName name="CTRL2general" hidden="0" function="0" vbProcedure="0">Contrôles!$L$32:$L$44</definedName>
     <definedName name="CTRL2type" hidden="0" function="0" vbProcedure="0">Contrôles!$J$32:$J$44</definedName>
     <definedName name="END_AVR" hidden="0" function="0" vbProcedure="0">Avoirs!$A$31</definedName>
@@ -5885,7 +5886,7 @@
       <c r="J32" s="370" t="n"/>
       <c r="K32" s="370" t="n"/>
       <c r="L32" s="370">
-        <f>ROUND(SUM(L4:L31),2)</f>
+        <f>ROUND(SUM(AVRmontant_solde_euro),2)</f>
         <v/>
       </c>
     </row>
@@ -7064,7 +7065,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="17.25" customHeight="1" s="290">
+    <row r="34" ht="16.5" customHeight="1" s="290">
       <c r="E34" s="416" t="inlineStr">
         <is>
           <t>-</t>
@@ -7385,7 +7386,7 @@
     <row r="1048512" ht="12.75" customHeight="1" s="290"/>
     <row r="1048513" ht="12.75" customHeight="1" s="290"/>
     <row r="1048514" ht="12.75" customHeight="1" s="290"/>
-    <row r="1048515" ht="12.75" customHeight="1" s="290"/>
+    <row r="1048515" ht="12.8" customHeight="1" s="290"/>
     <row r="1048516" ht="12.8" customHeight="1" s="290"/>
     <row r="1048517" ht="12.8" customHeight="1" s="290"/>
     <row r="1048518" ht="12.8" customHeight="1" s="290"/>

</xml_diff>

<commit_message>
feat: suppression 17 named ranges START/END du classeur DEV — named ranges colonnes seuls
</commit_message>
<xml_diff>
--- a/comptes_exemple.xlsx
+++ b/comptes_exemple.xlsx
@@ -62,14 +62,6 @@
     <definedName name="CTRL2eur" hidden="0" function="0" vbProcedure="0">Contrôles!$M$32:$M$44</definedName>
     <definedName name="CTRL2general" hidden="0" function="0" vbProcedure="0">Contrôles!$L$32:$L$44</definedName>
     <definedName name="CTRL2type" hidden="0" function="0" vbProcedure="0">Contrôles!$J$32:$J$44</definedName>
-    <definedName name="END_AVR" hidden="0" function="0" vbProcedure="0">Avoirs!$A$31</definedName>
-    <definedName name="END_CAT" hidden="0" function="0" vbProcedure="0">Budget!$E$35</definedName>
-    <definedName name="END_COT" hidden="0" function="0" vbProcedure="0">Cotations!$A$12</definedName>
-    <definedName name="END_CTRL1" hidden="0" function="0" vbProcedure="0">Contrôles!$A$26</definedName>
-    <definedName name="END_CTRL2" hidden="0" function="0" vbProcedure="0">Contrôles!$M$44</definedName>
-    <definedName name="END_PAT" hidden="0" function="0" vbProcedure="0">Patrimoine!$B$51</definedName>
-    <definedName name="END_POSTES" hidden="0" function="0" vbProcedure="0">Budget!$A$10</definedName>
-    <definedName name="END_PVL" hidden="0" function="0" vbProcedure="0">Plus_value!$B$52</definedName>
     <definedName name="OPcatégorie" hidden="0" function="0" vbProcedure="0">Opérations!$G$4:$G$10000</definedName>
     <definedName name="OPcommentaire" hidden="0" function="0" vbProcedure="0">Opérations!$I$4:$I$7193</definedName>
     <definedName name="OPcompte" hidden="0" function="0" vbProcedure="0">Opérations!$H$4:$H$10000</definedName>
@@ -98,15 +90,6 @@
     <definedName name="Retenu" hidden="0" function="0" vbProcedure="0">"Retenu"</definedName>
     <definedName name="Solde" hidden="0" function="0" vbProcedure="0">"#Solde"</definedName>
     <definedName name="Spéciale" hidden="0" function="0" vbProcedure="0">"#*"</definedName>
-    <definedName name="START_AVR" hidden="0" function="0" vbProcedure="0">Avoirs!$A$4</definedName>
-    <definedName name="START_CAT" hidden="0" function="0" vbProcedure="0">Budget!$E$19</definedName>
-    <definedName name="START_COT" hidden="0" function="0" vbProcedure="0">Cotations!$A$3</definedName>
-    <definedName name="START_CTRL1" hidden="0" function="0" vbProcedure="0">Contrôles!$A$3</definedName>
-    <definedName name="START_CTRL2" hidden="0" function="0" vbProcedure="0">Contrôles!$M$32</definedName>
-    <definedName name="START_OP" hidden="0" function="0" vbProcedure="0">Opérations!$A$4</definedName>
-    <definedName name="START_PAT" hidden="0" function="0" vbProcedure="0">Patrimoine!$B$5</definedName>
-    <definedName name="START_POSTES" hidden="0" function="0" vbProcedure="0">Budget!$A$4</definedName>
-    <definedName name="START_PVL" hidden="0" function="0" vbProcedure="0">Plus_value!$B$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Opérations'!$A$3:$I$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>

</xml_diff>

<commit_message>
fix: CTRL2 formules K/L étendues avec ajout devise
L(h+2) COMPTES : nouvelle formule SUM(EUR:last) — cohérence avec L(h+3/8/10)
K(h+2) COMPTES : IF(L=0) comme les autres K — plus de SUM inline
L(h+3) CATÉGORIES, L(h+8) € Virements, L(h+10) € Titres : SUM étendu
Suppression ÉTAPE F hardcodée (uno_col 16/17) remplacée par K/L named range
</commit_message>
<xml_diff>
--- a/comptes_exemple.xlsx
+++ b/comptes_exemple.xlsx
@@ -20478,11 +20478,12 @@
         </is>
       </c>
       <c r="K32" s="559">
-        <f>IF(SUM($L32:$M32)=0,"✓","✗")</f>
-        <v/>
-      </c>
-      <c r="L32" s="560" t="n">
-        <v>0</v>
+        <f>IF(L32=0,"✓","✗")</f>
+        <v/>
+      </c>
+      <c r="L32" s="560">
+        <f>SUM(M32:T32)</f>
+        <v/>
       </c>
       <c r="M32" s="560">
         <f>COUNTIFS($B3:$B26,M$30,$I3:$I26,"Oui")-COUNTIFS($B3:$B26,M$30,$I3:$I26,"Oui",$H3:$H26,0)</f>
@@ -20528,7 +20529,7 @@
         <v/>
       </c>
       <c r="L33" s="382">
-        <f>SUM(M33)</f>
+        <f>SUM(M33:T33)</f>
         <v/>
       </c>
       <c r="M33" s="382">
@@ -20730,7 +20731,7 @@
       </c>
       <c r="K38" s="317" t="n"/>
       <c r="L38" s="382">
-        <f>SUM(M38)</f>
+        <f>SUM(M38:T38)</f>
         <v/>
       </c>
       <c r="M38" s="382">
@@ -20815,7 +20816,7 @@
       </c>
       <c r="K40" s="317" t="n"/>
       <c r="L40" s="382">
-        <f>SUM(M40)</f>
+        <f>SUM(M40:T40)</f>
         <v/>
       </c>
       <c r="M40" s="382">

</xml_diff>

<commit_message>
Release v5.14.1 — ancrage PVL au premier #Solde (métaux/crypto/devises) : formule d'ancrage MAXIFS+OPequiv_euro (condition morte → epoch dégradé) corrigée en MINIFS (gui_devises Plus_value+Avoirs + tool_migrate_pvl_min_ancrage idempotent, sonde openpyxl bornée par named ranges). Fix rattrapage upgrade : pending_migrations joue TOUS les catchups idempotents (tri numérique via _version_tuple) au lieu du seul dernier. Value-neutral (TNR fast/build/example/light_build/pipe ✓). APP_VERSION 5.14.1, CHANGELOG, Compta_upgrade_classeur, Compta_pvl (re-ancrage = job de la purge). Exemple livré + 4 expected TNR migrés.
</commit_message>
<xml_diff>
--- a/comptes_exemple.xlsx
+++ b/comptes_exemple.xlsx
@@ -2880,7 +2880,7 @@
       <c r="E3" s="4"/>
       <c r="F3" s="5" t="str">
         <f aca="false">"dont Plus value latente depuis " &amp; YEAR(Plus_value!G3)</f>
-        <v>dont Plus value latente depuis 1899</v>
+        <v>dont Plus value latente depuis 2023</v>
       </c>
       <c r="G3" s="5"/>
       <c r="H3" s="8"/>
@@ -2902,11 +2902,11 @@
       <c r="F4" s="12"/>
       <c r="G4" s="11" t="n">
         <f aca="false">Plus_value!E3</f>
-        <v>415.0077973604</v>
+        <v>1455.0077973604</v>
       </c>
       <c r="H4" s="13" t="n">
         <f aca="false">Plus_value!F53</f>
-        <v>0.0790181430692849</v>
+        <v>0.345438765774654</v>
       </c>
       <c r="I4" s="13"/>
     </row>
@@ -4325,7 +4325,7 @@
         <v>43</v>
       </c>
       <c r="H6" s="57" t="n">
-        <f aca="false">_xlfn.MAXIFS(OPdate,OPcompte,$A6,OPdevise,$E6,OPcatégorie,Solde,OPequiv_euro,"&lt;&gt;")</f>
+        <f aca="false">_xlfn.MINIFS(OPdate,OPcompte,$A6,OPdevise,$E6,OPcatégorie,Solde)</f>
         <v>0</v>
       </c>
       <c r="I6" s="56" t="n">
@@ -4494,12 +4494,12 @@
         <v>43</v>
       </c>
       <c r="H10" s="57" t="n">
-        <f aca="false">_xlfn.MAXIFS(OPdate,OPcompte,$A10,OPdevise,$E10,OPcatégorie,Solde,OPequiv_euro,"&lt;&gt;")</f>
-        <v>0</v>
+        <f aca="false">_xlfn.MINIFS(OPdate,OPcompte,$A10,OPdevise,$E10,OPcatégorie,Solde)</f>
+        <v>45657</v>
       </c>
       <c r="I10" s="56" t="n">
         <f aca="false">SUMIFS(OPmontant,OPcompte,$A10,OPdevise,$E10,OPcatégorie,Solde,OPdate,$H10)</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J10" s="57" t="n">
         <f aca="false">_xlfn.MAXIFS(OPdate,OPcompte,$A10,OPdevise,$E10,OPcatégorie,Solde)</f>
@@ -4621,12 +4621,12 @@
         <v>42</v>
       </c>
       <c r="H13" s="57" t="n">
-        <f aca="false">_xlfn.MAXIFS(OPdate,OPcompte,$A13,OPdevise,$E13,OPcatégorie,Solde,OPequiv_euro,"&lt;&gt;")</f>
-        <v>0</v>
+        <f aca="false">_xlfn.MINIFS(OPdate,OPcompte,$A13,OPdevise,$E13,OPcatégorie,Solde)</f>
+        <v>45657</v>
       </c>
       <c r="I13" s="56" t="n">
         <f aca="false">SUMIFS(OPmontant,OPcompte,$A13,OPdevise,$E13,OPcatégorie,Solde,OPdate,$H13)</f>
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="J13" s="57" t="n">
         <f aca="false">_xlfn.MAXIFS(OPdate,OPcompte,$A13,OPdevise,$E13,OPcatégorie,Solde)</f>
@@ -4664,7 +4664,7 @@
         <v>43</v>
       </c>
       <c r="H14" s="57" t="n">
-        <f aca="false">_xlfn.MAXIFS(OPdate,OPcompte,$A14,OPdevise,$E14,OPcatégorie,Solde,OPequiv_euro,"&lt;&gt;")</f>
+        <f aca="false">_xlfn.MINIFS(OPdate,OPcompte,$A14,OPdevise,$E14,OPcatégorie,Solde)</f>
         <v>0</v>
       </c>
       <c r="I14" s="56" t="n">
@@ -4707,12 +4707,12 @@
         <v>43</v>
       </c>
       <c r="H15" s="57" t="n">
-        <f aca="false">_xlfn.MAXIFS(OPdate,OPcompte,$A15,OPdevise,$E15,OPcatégorie,Solde,OPequiv_euro,"&lt;&gt;")</f>
-        <v>0</v>
+        <f aca="false">_xlfn.MINIFS(OPdate,OPcompte,$A15,OPdevise,$E15,OPcatégorie,Solde)</f>
+        <v>46091</v>
       </c>
       <c r="I15" s="56" t="n">
         <f aca="false">SUMIFS(OPmontant,OPcompte,$A15,OPdevise,$E15,OPcatégorie,Solde,OPdate,$H15)</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J15" s="57" t="n">
         <f aca="false">_xlfn.MAXIFS(OPdate,OPcompte,$A15,OPdevise,$E15,OPcatégorie,Solde)</f>
@@ -4792,7 +4792,7 @@
         <v>43</v>
       </c>
       <c r="H17" s="57" t="n">
-        <f aca="false">_xlfn.MAXIFS(OPdate,OPcompte,$A17,OPdevise,$E17,OPcatégorie,Solde,OPequiv_euro,"&lt;&gt;")</f>
+        <f aca="false">_xlfn.MINIFS(OPdate,OPcompte,$A17,OPdevise,$E17,OPcatégorie,Solde)</f>
         <v>0</v>
       </c>
       <c r="I17" s="56" t="n">
@@ -4835,7 +4835,7 @@
         <v>43</v>
       </c>
       <c r="H18" s="57" t="n">
-        <f aca="false">_xlfn.MAXIFS(OPdate,OPcompte,$A18,OPdevise,$E18,OPcatégorie,Solde,OPequiv_euro,"&lt;&gt;")</f>
+        <f aca="false">_xlfn.MINIFS(OPdate,OPcompte,$A18,OPdevise,$E18,OPcatégorie,Solde)</f>
         <v>0</v>
       </c>
       <c r="I18" s="56" t="n">
@@ -4962,12 +4962,12 @@
         <v>43</v>
       </c>
       <c r="H21" s="57" t="n">
-        <f aca="false">_xlfn.MAXIFS(OPdate,OPcompte,$A21,OPdevise,$E21,OPcatégorie,Solde,OPequiv_euro,"&lt;&gt;")</f>
-        <v>0</v>
+        <f aca="false">_xlfn.MINIFS(OPdate,OPcompte,$A21,OPdevise,$E21,OPcatégorie,Solde)</f>
+        <v>45621</v>
       </c>
       <c r="I21" s="58" t="n">
         <f aca="false">SUMIFS(OPmontant,OPcompte,$A21,OPdevise,$E21,OPcatégorie,Solde,OPdate,$H21)</f>
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="J21" s="57" t="n">
         <f aca="false">_xlfn.MAXIFS(OPdate,OPcompte,$A21,OPdevise,$E21,OPcatégorie,Solde)</f>
@@ -5526,7 +5526,7 @@
       <c r="B1" s="12"/>
       <c r="C1" s="74" t="n">
         <f aca="false">C$2-365</f>
-        <v>45807</v>
+        <v>45845</v>
       </c>
       <c r="D1" s="74"/>
     </row>
@@ -5535,7 +5535,7 @@
       <c r="B2" s="12"/>
       <c r="C2" s="74" t="n">
         <f aca="true">TODAY()</f>
-        <v>46172</v>
+        <v>46210</v>
       </c>
       <c r="D2" s="74"/>
     </row>
@@ -5568,7 +5568,7 @@
       </c>
       <c r="C5" s="16" t="n">
         <f aca="false">SUMIF(CATposte,A5,CATaffectation)</f>
-        <v>-8.609095</v>
+        <v>-9.29126</v>
       </c>
       <c r="D5" s="16"/>
     </row>
@@ -5581,7 +5581,7 @@
       </c>
       <c r="C6" s="16" t="n">
         <f aca="false">SUMIF(CATposte,A6,CATaffectation)</f>
-        <v>9.161735</v>
+        <v>9.01494</v>
       </c>
       <c r="D6" s="16"/>
     </row>
@@ -5607,7 +5607,7 @@
       </c>
       <c r="C8" s="16" t="n">
         <f aca="false">SUMIF(CATposte,A8,CATaffectation)</f>
-        <v>-90</v>
+        <v>0</v>
       </c>
       <c r="D8" s="16"/>
     </row>
@@ -5639,7 +5639,7 @@
       <c r="B11" s="68"/>
       <c r="C11" s="71" t="n">
         <f aca="false">SUM(POSTESmontant)</f>
-        <v>-1879.44736</v>
+        <v>-1790.27632</v>
       </c>
       <c r="D11" s="76"/>
     </row>
@@ -5650,7 +5650,7 @@
       <c r="B12" s="78"/>
       <c r="C12" s="79" t="n">
         <f aca="false">SUMIF(POSTEStype,"Fixe",POSTESmontant)</f>
-        <v>-1879.44736</v>
+        <v>-1790.27632</v>
       </c>
       <c r="D12" s="80"/>
     </row>
@@ -5661,7 +5661,7 @@
       <c r="B13" s="78"/>
       <c r="C13" s="79" t="n">
         <f aca="false">C$12/12</f>
-        <v>-156.620613333333</v>
+        <v>-149.189693333333</v>
       </c>
       <c r="D13" s="81"/>
     </row>
@@ -5858,14 +5858,14 @@
       </c>
       <c r="G27" s="16" t="n">
         <f aca="false">SUMPRODUCT(SUMIFS(OPmontant,OPcatégorie,$E27,OPdate,"&gt;"&amp;$C$2-365,OPdevise,COTcode)*COTcours)</f>
-        <v>0.025905</v>
+        <v>-0.65626</v>
       </c>
       <c r="H27" s="92" t="n">
         <v>1</v>
       </c>
       <c r="I27" s="16" t="n">
         <f aca="false">G27*H27</f>
-        <v>0.025905</v>
+        <v>-0.65626</v>
       </c>
       <c r="J27" s="51" t="s">
         <v>120</v>
@@ -5881,14 +5881,14 @@
       </c>
       <c r="G28" s="16" t="n">
         <f aca="false">SUMPRODUCT(SUMIFS(OPmontant,OPcatégorie,$E28,OPdate,"&gt;"&amp;$C$2-365,OPdevise,COTcode)*COTcours)</f>
-        <v>9.161735</v>
+        <v>9.01494</v>
       </c>
       <c r="H28" s="92" t="n">
         <v>1</v>
       </c>
       <c r="I28" s="16" t="n">
         <f aca="false">G28*H28</f>
-        <v>9.161735</v>
+        <v>9.01494</v>
       </c>
       <c r="J28" s="51" t="s">
         <v>122</v>
@@ -6015,18 +6015,18 @@
       </c>
       <c r="F34" s="16" t="n">
         <f aca="false">SUMIFS(OPmontant,OPdevise,F$17,OPcatégorie,$E34,OPdate,"&gt;"&amp;$C$2-365)</f>
-        <v>-90</v>
+        <v>0</v>
       </c>
       <c r="G34" s="16" t="n">
         <f aca="false">SUMPRODUCT(SUMIFS(OPmontant,OPcatégorie,$E34,OPdate,"&gt;"&amp;$C$2-365,OPdevise,COTcode)*COTcours)</f>
-        <v>-90</v>
+        <v>0</v>
       </c>
       <c r="H34" s="92" t="n">
         <v>1</v>
       </c>
       <c r="I34" s="16" t="n">
         <f aca="false">G34*H34</f>
-        <v>-90</v>
+        <v>0</v>
       </c>
       <c r="J34" s="51" t="s">
         <v>124</v>
@@ -6048,11 +6048,11 @@
       </c>
       <c r="F36" s="71" t="n">
         <f aca="false">SUM(CATmontant)</f>
-        <v>-2898.08</v>
+        <v>-2808.08</v>
       </c>
       <c r="G36" s="71" t="n">
         <f aca="false">SUM(CATtotal_euro)</f>
-        <v>-1870.817225</v>
+        <v>-1781.646185</v>
       </c>
       <c r="H36" s="93"/>
       <c r="I36" s="71"/>
@@ -6064,11 +6064,11 @@
       </c>
       <c r="F37" s="79" t="n">
         <f aca="false">SUMIFS(OPmontant,OPdevise,F$17,OPdate,"&gt;"&amp;$C$2-365,OPcatégorie,"&lt;&gt;"&amp;Spéciale)</f>
-        <v>-2898.08</v>
+        <v>-2808.08</v>
       </c>
       <c r="G37" s="79" t="n">
         <f aca="false">SUMPRODUCT(SUMIFS(OPmontant,OPdate,"&gt;"&amp;$C$2-365,OPcatégorie,"&lt;&gt;"&amp;Spéciale,OPdevise,COTcode)*COTcours)</f>
-        <v>-1870.817225</v>
+        <v>-1781.646185</v>
       </c>
       <c r="H37" s="94"/>
       <c r="I37" s="79"/>
@@ -6096,16 +6096,16 @@
       </c>
       <c r="F39" s="79" t="n">
         <f aca="false">SUMIFS(CATmontant,CATnom,"&lt;&gt;@*")</f>
-        <v>-1880</v>
+        <v>-1790</v>
       </c>
       <c r="G39" s="79" t="n">
         <f aca="false">SUMIFS(CATtotal_euro,CATnom,"&lt;&gt;@*")</f>
-        <v>-1879.44736</v>
+        <v>-1790.27632</v>
       </c>
       <c r="H39" s="94"/>
       <c r="I39" s="79" t="n">
         <f aca="false">SUMIFS(CATaffectation,CATnom,"&lt;&gt;@*")</f>
-        <v>-1879.44736</v>
+        <v>-1790.27632</v>
       </c>
       <c r="J39" s="94"/>
     </row>
@@ -6115,11 +6115,11 @@
       </c>
       <c r="F40" s="79" t="n">
         <f aca="false">F$39*INDEX(COTcours,MATCH($F$17,COTcode,0))</f>
-        <v>-1880</v>
+        <v>-1790</v>
       </c>
       <c r="G40" s="79" t="n">
         <f aca="false">SUM(F$40)</f>
-        <v>-1880</v>
+        <v>-1790</v>
       </c>
       <c r="H40" s="94"/>
       <c r="I40" s="79"/>
@@ -6372,12 +6372,12 @@
       <c r="D3" s="84"/>
       <c r="E3" s="11" t="n">
         <f aca="false">E53</f>
-        <v>415.0077973604</v>
+        <v>1455.0077973604</v>
       </c>
       <c r="F3" s="84"/>
       <c r="G3" s="96" t="n">
         <f aca="false">G53</f>
-        <v>0</v>
+        <v>44927</v>
       </c>
       <c r="H3" s="46"/>
       <c r="I3" s="12"/>
@@ -7382,12 +7382,12 @@
       </c>
       <c r="E39" s="101" t="n">
         <f aca="false">K39-(H39+I39)</f>
-        <v>1128.4858754304</v>
+        <v>2118.4858754304</v>
       </c>
       <c r="F39" s="51"/>
       <c r="G39" s="102" t="n">
-        <f aca="false">_xlfn.MAXIFS(OPdate,OPcompte,B39,OPdevise,D39,OPcatégorie,Solde,OPequiv_euro,"&lt;&gt;")</f>
-        <v>0</v>
+        <f aca="false">_xlfn.MINIFS(OPdate,OPcompte,B39,OPdevise,D39,OPcatégorie,Solde)</f>
+        <v>45457</v>
       </c>
       <c r="H39" s="103" t="n">
         <f aca="false">SUMIFS(OPequiv_euro,OPcompte,B39,OPdevise,D39,OPcatégorie,Solde,OPdate,G39)</f>
@@ -7395,7 +7395,7 @@
       </c>
       <c r="I39" s="103" t="n">
         <f aca="false">SUMIFS(OPequiv_euro,OPcompte,B39,OPdevise,D39,OPcatégorie,"&lt;&gt;"&amp;Spéciale,OPdate,"&gt;="&amp;G39)</f>
-        <v>990</v>
+        <v>0</v>
       </c>
       <c r="J39" s="102" t="n">
         <f aca="false">SUMIF(AVRintitulé,$B39,AVRdate_solde)</f>
@@ -7451,8 +7451,8 @@
       </c>
       <c r="F42" s="51"/>
       <c r="G42" s="102" t="n">
-        <f aca="false">_xlfn.MAXIFS(OPdate,OPcompte,B42,OPdevise,D42,OPcatégorie,Solde,OPequiv_euro,"&lt;&gt;")</f>
-        <v>0</v>
+        <f aca="false">_xlfn.MINIFS(OPdate,OPcompte,B42,OPdevise,D42,OPcatégorie,Solde)</f>
+        <v>44927</v>
       </c>
       <c r="H42" s="103" t="n">
         <f aca="false">SUMIFS(OPequiv_euro,OPcompte,B42,OPdevise,D42,OPcatégorie,Solde,OPdate,G42)</f>
@@ -7484,12 +7484,12 @@
       </c>
       <c r="E43" s="101" t="n">
         <f aca="false">K43-(H43+I43)</f>
-        <v>120.093092</v>
+        <v>170.093092</v>
       </c>
       <c r="F43" s="51"/>
       <c r="G43" s="102" t="n">
-        <f aca="false">_xlfn.MAXIFS(OPdate,OPcompte,B43,OPdevise,D43,OPcatégorie,Solde,OPequiv_euro,"&lt;&gt;")</f>
-        <v>0</v>
+        <f aca="false">_xlfn.MINIFS(OPdate,OPcompte,B43,OPdevise,D43,OPcatégorie,Solde)</f>
+        <v>45292</v>
       </c>
       <c r="H43" s="103" t="n">
         <f aca="false">SUMIFS(OPequiv_euro,OPcompte,B43,OPdevise,D43,OPcatégorie,Solde,OPdate,G43)</f>
@@ -7497,7 +7497,7 @@
       </c>
       <c r="I43" s="103" t="n">
         <f aca="false">SUMIFS(OPequiv_euro,OPcompte,B43,OPdevise,D43,OPcatégorie,"&lt;&gt;"&amp;Spéciale,OPdate,"&gt;="&amp;G43)</f>
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="J43" s="102" t="n">
         <f aca="false">SUMIF(AVRintitulé,$B43,AVRdate_solde)</f>
@@ -7525,8 +7525,8 @@
       </c>
       <c r="F44" s="51"/>
       <c r="G44" s="102" t="n">
-        <f aca="false">_xlfn.MAXIFS(OPdate,OPcompte,B44,OPdevise,D44,OPcatégorie,Solde,OPequiv_euro,"&lt;&gt;")</f>
-        <v>0</v>
+        <f aca="false">_xlfn.MINIFS(OPdate,OPcompte,B44,OPdevise,D44,OPcatégorie,Solde)</f>
+        <v>45923</v>
       </c>
       <c r="H44" s="103" t="n">
         <f aca="false">SUMIFS(OPequiv_euro,OPcompte,B44,OPdevise,D44,OPcatégorie,Solde,OPdate,G44)</f>
@@ -7562,7 +7562,7 @@
       </c>
       <c r="F45" s="51"/>
       <c r="G45" s="102" t="n">
-        <f aca="false">_xlfn.MAXIFS(OPdate,OPcompte,B45,OPdevise,D45,OPcatégorie,Solde,OPequiv_euro,"&lt;&gt;")</f>
+        <f aca="false">_xlfn.MINIFS(OPdate,OPcompte,B45,OPdevise,D45,OPcatégorie,Solde)</f>
         <v>0</v>
       </c>
       <c r="H45" s="103" t="n">
@@ -7627,7 +7627,7 @@
       </c>
       <c r="F48" s="51"/>
       <c r="G48" s="102" t="n">
-        <f aca="false">_xlfn.MAXIFS(OPdate,OPcompte,B48,OPdevise,D48,OPcatégorie,Solde,OPequiv_euro,"&lt;&gt;")</f>
+        <f aca="false">_xlfn.MINIFS(OPdate,OPcompte,B48,OPdevise,D48,OPcatégorie,Solde)</f>
         <v>0</v>
       </c>
       <c r="H48" s="103" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="F49" s="51"/>
       <c r="G49" s="102" t="n">
-        <f aca="false">_xlfn.MAXIFS(OPdate,OPcompte,B49,OPdevise,D49,OPcatégorie,Solde,OPequiv_euro,"&lt;&gt;")</f>
+        <f aca="false">_xlfn.MINIFS(OPdate,OPcompte,B49,OPdevise,D49,OPcatégorie,Solde)</f>
         <v>0</v>
       </c>
       <c r="H49" s="103" t="n">
@@ -7701,8 +7701,8 @@
       </c>
       <c r="F50" s="51"/>
       <c r="G50" s="102" t="n">
-        <f aca="false">_xlfn.MAXIFS(OPdate,OPcompte,B50,OPdevise,D50,OPcatégorie,Solde,OPequiv_euro,"&lt;&gt;")</f>
-        <v>0</v>
+        <f aca="false">_xlfn.MINIFS(OPdate,OPcompte,B50,OPdevise,D50,OPcatégorie,Solde)</f>
+        <v>45621</v>
       </c>
       <c r="H50" s="103" t="n">
         <f aca="false">SUMIFS(OPequiv_euro,OPcompte,B50,OPdevise,D50,OPcatégorie,Solde,OPdate,G50)</f>
@@ -7760,15 +7760,15 @@
       </c>
       <c r="E53" s="117" t="n">
         <f aca="false">SUM(E54:E57)</f>
-        <v>415.0077973604</v>
+        <v>1455.0077973604</v>
       </c>
       <c r="F53" s="118" t="n">
         <f aca="false">E53/(H53+I53)</f>
-        <v>0.0790181430692849</v>
+        <v>0.345438765774654</v>
       </c>
       <c r="G53" s="119" t="n">
         <f aca="false">MIN(G54:G57)</f>
-        <v>0</v>
+        <v>44927</v>
       </c>
       <c r="H53" s="120" t="n">
         <f aca="false">SUM(H54:H57)</f>
@@ -7776,7 +7776,7 @@
       </c>
       <c r="I53" s="120" t="n">
         <f aca="false">SUM(I54:I57)</f>
-        <v>2187.12427</v>
+        <v>1147.12427</v>
       </c>
       <c r="J53" s="121"/>
       <c r="K53" s="117" t="n">
@@ -7833,15 +7833,15 @@
       </c>
       <c r="E55" s="122" t="n">
         <f aca="false">K55-(H55+I55)</f>
-        <v>1128.4858754304</v>
-      </c>
-      <c r="F55" s="123" t="n">
+        <v>2118.4858754304</v>
+      </c>
+      <c r="F55" s="123" t="e">
         <f aca="false">E55/(H55+I55)</f>
-        <v>1.13988472265697</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G55" s="124" t="n">
         <f aca="false">MIN(_xlfn.MINIFS(G:G,A:A,"métaux",G:G,"&gt;0"))</f>
-        <v>0</v>
+        <v>45457</v>
       </c>
       <c r="H55" s="125" t="n">
         <f aca="false">SUMIFS(PVLmontant_init,PVLsection,"métaux")</f>
@@ -7849,7 +7849,7 @@
       </c>
       <c r="I55" s="125" t="n">
         <f aca="false">SUMIFS(PVLsigma,PVLsection,"métaux")</f>
-        <v>990</v>
+        <v>0</v>
       </c>
       <c r="J55" s="124" t="n">
         <f aca="false">_xlfn.MAXIFS(J:J,A:A,"métaux")</f>
@@ -7871,15 +7871,15 @@
       </c>
       <c r="E56" s="122" t="n">
         <f aca="false">K56-(H56+I56)</f>
-        <v>251.37667693</v>
+        <v>301.37667693</v>
       </c>
       <c r="F56" s="123" t="n">
         <f aca="false">E56/(H56+I56)</f>
-        <v>-5.0275335386</v>
+        <v>-3.0137667693</v>
       </c>
       <c r="G56" s="124" t="n">
         <f aca="false">MIN(_xlfn.MINIFS(G:G,A:A,"crypto",G:G,"&gt;0"))</f>
-        <v>0</v>
+        <v>44927</v>
       </c>
       <c r="H56" s="125" t="n">
         <f aca="false">SUMIFS(PVLmontant_init,PVLsection,"crypto")</f>
@@ -7887,7 +7887,7 @@
       </c>
       <c r="I56" s="125" t="n">
         <f aca="false">SUMIFS(PVLsigma,PVLsection,"crypto")</f>
-        <v>-50</v>
+        <v>-100</v>
       </c>
       <c r="J56" s="124" t="n">
         <f aca="false">_xlfn.MAXIFS(J:J,A:A,"crypto")</f>
@@ -7917,7 +7917,7 @@
       </c>
       <c r="G57" s="124" t="n">
         <f aca="false">MIN(_xlfn.MINIFS(G:G,A:A,"devises",G:G,"&gt;0"))</f>
-        <v>0</v>
+        <v>45621</v>
       </c>
       <c r="H57" s="125" t="n">
         <f aca="false">SUMIFS(PVLmontant_init,PVLsection,"devises")</f>
@@ -8082,7 +8082,7 @@
     <row r="2" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="128" t="n">
         <f aca="true">TODAY()</f>
-        <v>46172</v>
+        <v>46210</v>
       </c>
       <c r="B2" s="48" t="str">
         <f aca="false">Contrôles!K$49</f>

</xml_diff>

<commit_message>
CLAUDE s.214 : #176 BALANCES ROUND livré (migration catchup 3→3 tool_migrate_ctrl_changes_round + template/exemple + upgrade_map/docs) ; #177 audit 11 fetchers → 3 corrigés (ETORO finally/override/force ; SOCGEN _fail×11 ; DEGIRO download_csv) ; release v5.22.0 (APP_VERSION + CHANGELOG + upgrade)
</commit_message>
<xml_diff>
--- a/comptes_exemple.xlsx
+++ b/comptes_exemple.xlsx
@@ -1030,7 +1030,7 @@
     <numFmt numFmtId="204" formatCode="#,##0.000000000\ [$USD]"/>
     <numFmt numFmtId="205" formatCode="#,##0.000000000\ [$SGD]"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1124,13 +1124,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF0432FF"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -1754,7 +1747,7 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="13" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1762,15 +1755,15 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="16" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="16" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1882,7 +1875,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1922,7 +1915,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="16" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="18" fillId="16" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1970,7 +1963,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1978,11 +1971,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="16" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="17" fillId="16" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="178" fontId="20" fillId="16" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="178" fontId="19" fillId="16" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2094,7 +2087,7 @@
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="195" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="195" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2114,7 +2107,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="195" fontId="17" fillId="18" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="195" fontId="16" fillId="18" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2150,7 +2143,7 @@
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="16" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="18" fillId="16" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2178,7 +2171,7 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="197" fontId="17" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="197" fontId="16" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2262,7 +2255,7 @@
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5578,7 +5571,7 @@
       <c r="B1" s="12"/>
       <c r="C1" s="75" t="n">
         <f aca="false">C$2-365</f>
-        <v>45847</v>
+        <v>45857</v>
       </c>
       <c r="D1" s="75"/>
     </row>
@@ -5587,7 +5580,7 @@
       <c r="B2" s="12"/>
       <c r="C2" s="75" t="n">
         <f aca="true">TODAY()</f>
-        <v>46212</v>
+        <v>46222</v>
       </c>
       <c r="D2" s="75"/>
     </row>
@@ -8134,7 +8127,7 @@
     <row r="2" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="129" t="n">
         <f aca="true">TODAY()</f>
-        <v>46212</v>
+        <v>46222</v>
       </c>
       <c r="B2" s="49" t="str">
         <f aca="false">Contrôles!K$49</f>
@@ -18288,7 +18281,7 @@
       </c>
       <c r="K42" s="55"/>
       <c r="L42" s="91" t="n">
-        <f aca="false">SUMIFS(OPequiv_euro,OPcatégorie,"@Change") + SUMIFS(OPequiv_euro,OPcatégorie,"@Achat métaux")</f>
+        <f aca="false">ROUND(SUMIFS(OPequiv_euro,OPcatégorie,"@Change") + SUMIFS(OPequiv_euro,OPcatégorie,"@Achat métaux"),0)</f>
         <v>0</v>
       </c>
       <c r="M42" s="104" t="n">

</xml_diff>